<commit_message>
move into supporting info folder
</commit_message>
<xml_diff>
--- a/Supporting Info/show_genres.xlsx
+++ b/Supporting Info/show_genres.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Henry\Documents\GitHub Repos\Japanese-Similarity-Analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Henry\Documents\GitHub Repos\Japanese-Similarity-Analysis\Supporting Info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B78C9B18-06EB-4535-8F37-5355EE44AD29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F5F76E1-B0E8-4344-A3C3-5DC2FFD406BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="11640" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21830" yWindow="6440" windowWidth="15450" windowHeight="9300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -365,9 +365,6 @@
     <t>Suspense</t>
   </si>
   <si>
-    <t>Slice of Life</t>
-  </si>
-  <si>
     <t>Action, Mystery, Supernatural</t>
   </si>
   <si>
@@ -392,9 +389,6 @@
     <t>Action, Fantasy, Sci-Fi</t>
   </si>
   <si>
-    <t>Slice of Life, Supernatural</t>
-  </si>
-  <si>
     <t>Drama, Romance, Supernatural</t>
   </si>
   <si>
@@ -407,36 +401,24 @@
     <t>Action, Adventure, Mystery</t>
   </si>
   <si>
-    <t>Mystery, Slice of Life</t>
-  </si>
-  <si>
     <t>Mystery, Sci-Fi, Suspense</t>
   </si>
   <si>
     <t>Comedy, Drama, Mystery</t>
   </si>
   <si>
-    <t>Fantasy, Slice of Life</t>
-  </si>
-  <si>
     <t>Adventure, Comedy, Romance</t>
   </si>
   <si>
     <t>Drama, Fantasy, Romance</t>
   </si>
   <si>
-    <t>Avant Garde, Drama, Mystery, Supernatural</t>
-  </si>
-  <si>
     <t>Avant Garde</t>
   </si>
   <si>
     <t>Sci-Fi, Sports</t>
   </si>
   <si>
-    <t>Adventure, Mystery, Slice of Life, Supernatural</t>
-  </si>
-  <si>
     <t>Adventure, Sci-Fi</t>
   </si>
   <si>
@@ -470,9 +452,6 @@
     <t>Mystery, Supernatural, Suspense</t>
   </si>
   <si>
-    <t>Romance, Slice of Life</t>
-  </si>
-  <si>
     <t>Comedy, Mystery, Romance</t>
   </si>
   <si>
@@ -527,18 +506,12 @@
     <t>Aho-Girl</t>
   </si>
   <si>
-    <t>Ao-no-hako</t>
-  </si>
-  <si>
     <t>Romance, Sports</t>
   </si>
   <si>
     <t>Sket-Dance</t>
   </si>
   <si>
-    <t>Higashi-no-eden</t>
-  </si>
-  <si>
     <t>Mystery, Romance, Sci-Fi, Suspense</t>
   </si>
   <si>
@@ -564,6 +537,33 @@
   </si>
   <si>
     <t>Non-non-biyori</t>
+  </si>
+  <si>
+    <t>Slice-of-Life</t>
+  </si>
+  <si>
+    <t>Slice-of-Life, Supernatural</t>
+  </si>
+  <si>
+    <t>Mystery, Slice-of-Life</t>
+  </si>
+  <si>
+    <t>Fantasy, Slice-of-Life</t>
+  </si>
+  <si>
+    <t>Adventure, Mystery, Slice-of-Life, Supernatural</t>
+  </si>
+  <si>
+    <t>Romance, Slice-of-Life</t>
+  </si>
+  <si>
+    <t>Avant-Garde, Drama, Mystery, Supernatural</t>
+  </si>
+  <si>
+    <t>Ao-no-Hako</t>
+  </si>
+  <si>
+    <t>Higashi-no-Eden</t>
   </si>
 </sst>
 </file>
@@ -953,7 +953,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>89</v>
@@ -962,7 +962,7 @@
         <v>2020</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="G3" t="s">
         <v>90</v>
@@ -1058,7 +1058,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>89</v>
@@ -1079,7 +1079,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>89</v>
@@ -1121,7 +1121,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>89</v>
@@ -1130,10 +1130,10 @@
         <v>2022</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>109</v>
+        <v>167</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H11">
         <f>COUNTIF($D:$D, "*Supernatural*")</f>
@@ -1154,16 +1154,16 @@
         <v>102</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>109</v>
+        <v>167</v>
       </c>
       <c r="H12">
-        <f>COUNTIF($D:$D, "*Slice of Life*")</f>
+        <f>COUNTIF($D:$D, "*Slice-of-Life*")</f>
         <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>89</v>
@@ -1172,7 +1172,7 @@
         <v>2024</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>108</v>
@@ -1196,7 +1196,7 @@
         <v>103</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H14">
         <f>COUNTIF($D:$D, "*Ecchi*")</f>
@@ -1217,10 +1217,10 @@
         <v>104</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="H15">
-        <f>COUNTIF($D:$D, "*Avant Garde*")</f>
+        <f>COUNTIF($D:$D, "*Avant-Garde*")</f>
         <v>1</v>
       </c>
     </row>
@@ -1278,12 +1278,12 @@
         <v>2014</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>109</v>
+        <v>167</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>89</v>
@@ -1292,7 +1292,7 @@
         <v>2019</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -1339,7 +1339,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>89</v>
@@ -1348,7 +1348,7 @@
         <v>2016</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
@@ -1376,7 +1376,7 @@
         <v>2016</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
@@ -1432,7 +1432,7 @@
         <v>2011</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
@@ -1451,7 +1451,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>89</v>
@@ -1460,7 +1460,7 @@
         <v>2006</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -1474,7 +1474,7 @@
         <v>2020</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
@@ -1488,7 +1488,7 @@
         <v>2020</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -1502,7 +1502,7 @@
         <v>2019</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -1516,7 +1516,7 @@
         <v>2021</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
@@ -1530,7 +1530,7 @@
         <v>2019</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -1544,7 +1544,7 @@
         <v>2016</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>118</v>
+        <v>168</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -1572,7 +1572,7 @@
         <v>2019</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
@@ -1600,7 +1600,7 @@
         <v>2010</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -1614,7 +1614,7 @@
         <v>2020</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
@@ -1628,12 +1628,12 @@
         <v>2020</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>89</v>
@@ -1661,7 +1661,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>89</v>
@@ -1670,7 +1670,7 @@
         <v>2009</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
@@ -1698,7 +1698,7 @@
         <v>2012</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>123</v>
+        <v>169</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
@@ -1712,7 +1712,7 @@
         <v>2020</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
@@ -1726,7 +1726,7 @@
         <v>2015</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
@@ -1754,7 +1754,7 @@
         <v>2019</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
@@ -1768,7 +1768,7 @@
         <v>2018</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
@@ -1782,7 +1782,7 @@
         <v>2017</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>126</v>
+        <v>170</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
@@ -1838,7 +1838,7 @@
         <v>2014</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
@@ -1852,7 +1852,7 @@
         <v>2017</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
@@ -1880,7 +1880,7 @@
         <v>2011</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>129</v>
+        <v>173</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
@@ -1894,7 +1894,7 @@
         <v>2018</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
@@ -1908,7 +1908,7 @@
         <v>2005</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>132</v>
+        <v>171</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
@@ -1922,12 +1922,12 @@
         <v>2013</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>89</v>
@@ -1936,7 +1936,7 @@
         <v>2008</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>118</v>
+        <v>168</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
@@ -1950,7 +1950,7 @@
         <v>2019</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
@@ -1964,7 +1964,7 @@
         <v>2022</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
@@ -1978,7 +1978,7 @@
         <v>2022</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
@@ -1992,7 +1992,7 @@
         <v>2021</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
@@ -2006,7 +2006,7 @@
         <v>2003</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
@@ -2020,7 +2020,7 @@
         <v>2020</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
@@ -2034,7 +2034,7 @@
         <v>2017</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
@@ -2048,7 +2048,7 @@
         <v>2012</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
@@ -2062,12 +2062,12 @@
         <v>2016</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>89</v>
@@ -2076,7 +2076,7 @@
         <v>2016</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
@@ -2104,7 +2104,7 @@
         <v>2014</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
@@ -2118,12 +2118,12 @@
         <v>2018</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>89</v>
@@ -2174,7 +2174,7 @@
         <v>2012</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
@@ -2188,7 +2188,7 @@
         <v>2022</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
@@ -2202,7 +2202,7 @@
         <v>2021</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
@@ -2216,7 +2216,7 @@
         <v>2016</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
@@ -2230,12 +2230,12 @@
         <v>2014</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>144</v>
+        <v>172</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>89</v>
@@ -2244,7 +2244,7 @@
         <v>2016</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>109</v>
+        <v>167</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
@@ -2258,7 +2258,7 @@
         <v>2021</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
@@ -2272,7 +2272,7 @@
         <v>2012</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
@@ -2286,7 +2286,7 @@
         <v>2011</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>109</v>
+        <v>167</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
@@ -2300,7 +2300,7 @@
         <v>2021</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.35">
@@ -2314,7 +2314,7 @@
         <v>2019</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.35">
@@ -2328,7 +2328,7 @@
         <v>2018</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
@@ -2342,7 +2342,7 @@
         <v>2021</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
@@ -2370,12 +2370,12 @@
         <v>2019</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>89</v>
@@ -2384,7 +2384,7 @@
         <v>2022</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
@@ -2412,12 +2412,12 @@
         <v>2018</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>109</v>
+        <v>167</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>89</v>
@@ -2426,7 +2426,7 @@
         <v>2013</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>109</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>